<commit_message>
demo-at: build triggered by rockphotog for commit 59c3dcbdb87ffa525503618a6351ec5dce1e10cb 59c3dcbdb87ffa525503618a6351ec5dce1e10cb
</commit_message>
<xml_diff>
--- a/currentbuild/ValueSet-annen-allergi-som-kritisk-informasjon-7514.xlsx
+++ b/currentbuild/ValueSet-annen-allergi-som-kritisk-informasjon-7514.xlsx
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-15T12:51:38+00:00</t>
+    <t>2026-09-15T13:41:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>